<commit_message>
Actualización automática 2026-01-08 15:30:09
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -2340,7 +2340,7 @@
         <v>0</v>
       </c>
       <c r="M31" s="2" t="n">
-        <v>1496.72</v>
+        <v>1694.28</v>
       </c>
       <c r="N31" s="2" t="n">
         <v>0</v>
@@ -4984,7 +4984,7 @@
         <v>0</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>1496.72</v>
+        <v>1694.28</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>0</v>
@@ -5757,7 +5757,7 @@
         <v>57170.26</v>
       </c>
       <c r="F60" s="6" t="n">
-        <v>11393.66</v>
+        <v>11591.22</v>
       </c>
       <c r="G60" s="6" t="n">
         <v>47000</v>

</xml_diff>

<commit_message>
Actualización automática 2026-01-09 17:30:07
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -900,7 +900,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>14685.95</v>
+        <v>22781.83</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -2956,7 +2956,7 @@
         <v>6961.7</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>14685.95</v>
+        <v>22781.83</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>10000</v>
@@ -3756,7 +3756,7 @@
         <v>38735.68</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>20779.01</v>
+        <v>28874.89</v>
       </c>
       <c r="G37" s="6" t="n">
         <v>35500</v>

</xml_diff>

<commit_message>
Actualización automática 2026-01-20 17:30:12
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -600,7 +600,7 @@
         <v>0</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>0</v>
+        <v>1711.22</v>
       </c>
       <c r="N2" s="2" t="n">
         <v>0</v>
@@ -2711,7 +2711,7 @@
       </c>
       <c r="M37" s="4" t="inlineStr">
         <is>
-          <t>3 de 35</t>
+          <t>4 de 35</t>
         </is>
       </c>
       <c r="N37" s="4" t="inlineStr">
@@ -2821,7 +2821,7 @@
         <v>4877.83</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0</v>
+        <v>1711.22</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>2000</v>
@@ -3756,7 +3756,7 @@
         <v>38735.68</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>29022.19</v>
+        <v>30733.41</v>
       </c>
       <c r="G37" s="6" t="n">
         <v>35500</v>
@@ -3779,8 +3779,8 @@
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -4071,13 +4071,13 @@
         <v>37250</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>27583.7</v>
+        <v>29294.92</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>9666.299999999999</v>
+        <v>7955.080000000002</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.7405020134228188</v>
+        <v>0.7864408053691274</v>
       </c>
     </row>
     <row r="13">
@@ -4138,13 +4138,13 @@
         <v>46287.26300000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>34749.31</v>
+        <v>36460.53</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>11537.953</v>
+        <v>9826.733</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.7507315781449422</v>
+        <v>0.7877011436169815</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-01-22 10:30:11
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -1740,7 +1740,7 @@
         <v>0</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>0</v>
+        <v>29.44</v>
       </c>
       <c r="N21" s="2" t="n">
         <v>0</v>
@@ -2711,7 +2711,7 @@
       </c>
       <c r="M37" s="4" t="inlineStr">
         <is>
-          <t>4 de 35</t>
+          <t>5 de 35</t>
         </is>
       </c>
       <c r="N37" s="4" t="inlineStr">
@@ -3334,7 +3334,7 @@
         <v>0</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0</v>
+        <v>29.44</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>2500</v>
@@ -3756,7 +3756,7 @@
         <v>38735.68</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>31961.57</v>
+        <v>31991.01</v>
       </c>
       <c r="G37" s="6" t="n">
         <v>35500</v>
@@ -3780,7 +3780,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -4071,13 +4071,13 @@
         <v>37250</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>30523.08</v>
+        <v>30552.52</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>6726.919999999998</v>
+        <v>6697.48</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.8194115436241611</v>
+        <v>0.8202018791946308</v>
       </c>
     </row>
     <row r="13">
@@ -4138,13 +4138,13 @@
         <v>46287.26300000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>37688.69</v>
+        <v>37718.13</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>8598.572999999997</v>
+        <v>8569.132999999998</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.8142345767992374</v>
+        <v>0.8148706049005316</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-01-26 10:30:13
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -3780,7 +3780,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -4071,13 +4071,13 @@
         <v>37250</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>30552.52</v>
+        <v>30581.96</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>6697.48</v>
+        <v>6668.040000000001</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.8202018791946308</v>
+        <v>0.8209922147651006</v>
       </c>
     </row>
     <row r="13">
@@ -4138,13 +4138,13 @@
         <v>46287.26300000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>37718.13</v>
+        <v>37747.56999999999</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>8569.132999999998</v>
+        <v>8539.692999999999</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.8148706049005316</v>
+        <v>0.8155066330018257</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-01-29 12:30:14
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -1728,7 +1728,7 @@
         <v>0</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>0</v>
+        <v>1902.56</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0</v>
@@ -2691,7 +2691,7 @@
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>1 de 35</t>
+          <t>2 de 35</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3334,7 +3334,7 @@
         <v>0</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>29.44</v>
+        <v>1932</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>2500</v>
@@ -3756,7 +3756,7 @@
         <v>38735.68</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>31991.01</v>
+        <v>33893.57000000001</v>
       </c>
       <c r="G37" s="6" t="n">
         <v>35500</v>
@@ -3951,13 +3951,13 @@
         <v>916.65</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>364.5</v>
+        <v>2267.06</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>552.15</v>
+        <v>-1350.41</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.3976435935198822</v>
+        <v>2.47320133093329</v>
       </c>
     </row>
     <row r="8">
@@ -4162,13 +4162,13 @@
         <v>46747.26300000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>37635.69</v>
+        <v>39538.25</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>9111.572999999997</v>
+        <v>7209.012999999997</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.8050886316060899</v>
+        <v>0.8457874849271924</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-01-29 15:30:12
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -1860,7 +1860,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>0</v>
+        <v>14.76</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -2711,7 +2711,7 @@
       </c>
       <c r="M37" s="4" t="inlineStr">
         <is>
-          <t>5 de 35</t>
+          <t>6 de 35</t>
         </is>
       </c>
       <c r="N37" s="4" t="inlineStr">
@@ -3388,7 +3388,7 @@
         <v>126.72</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0</v>
+        <v>14.76</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>1000</v>
@@ -3756,7 +3756,7 @@
         <v>38735.68</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>33893.57000000001</v>
+        <v>33908.33</v>
       </c>
       <c r="G37" s="6" t="n">
         <v>35500</v>
@@ -3780,7 +3780,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -4095,13 +4095,13 @@
         <v>37250</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>30470.08</v>
+        <v>30484.84</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>6779.919999999998</v>
+        <v>6765.16</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.8179887248322149</v>
+        <v>0.818384966442953</v>
       </c>
     </row>
     <row r="14">
@@ -4162,13 +4162,13 @@
         <v>46747.26300000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>39538.25</v>
+        <v>39553.00999999999</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>7209.012999999997</v>
+        <v>7194.252999999999</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.8457874849271924</v>
+        <v>0.8461032253374917</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-05 17:30:21
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -993,7 +993,7 @@
         <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>5037.12</v>
+        <v>8700.48</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0</v>
@@ -1020,7 +1020,7 @@
         <v>0</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>2601.72</v>
+        <v>7924.3</v>
       </c>
       <c r="N9" s="2" t="n">
         <v>0</v>
@@ -2759,7 +2759,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3010,7 +3010,7 @@
         <v>0</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>7638.84</v>
+        <v>16624.78</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>14000</v>
@@ -3756,7 +3756,7 @@
         <v>35073.75000000001</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>7665.84</v>
+        <v>16651.78</v>
       </c>
       <c r="G37" s="6" t="n">
         <v>35500</v>
@@ -3781,7 +3781,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3855,13 +3855,13 @@
         <v>1514</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>5037.12</v>
+        <v>8700.48</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-3523.12</v>
+        <v>-7186.48</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>3.327027741083223</v>
+        <v>5.74668428005284</v>
       </c>
     </row>
     <row r="4">
@@ -4095,13 +4095,13 @@
         <v>35250</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>2628.72</v>
+        <v>7951.3</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>32621.28</v>
+        <v>27298.7</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.07457361702127659</v>
+        <v>0.2255687943262411</v>
       </c>
     </row>
     <row r="14">
@@ -4162,13 +4162,13 @@
         <v>43747.113</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>7665.84</v>
+        <v>16651.78</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>36081.273</v>
+        <v>27095.333</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.1752307632277357</v>
+        <v>0.380637231992886</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-05 10:30:19
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -597,10 +597,10 @@
         <v>0</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>0</v>
+        <v>380.16</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>0</v>
+        <v>2281.62</v>
       </c>
       <c r="N2" s="2" t="n">
         <v>0</v>
@@ -2706,12 +2706,12 @@
       </c>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>0 de 35</t>
+          <t>1 de 35</t>
         </is>
       </c>
       <c r="M37" s="4" t="inlineStr">
         <is>
-          <t>0 de 35</t>
+          <t>1 de 35</t>
         </is>
       </c>
       <c r="N37" s="4" t="inlineStr">
@@ -2759,7 +2759,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -2821,7 +2821,7 @@
         <v>0</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0</v>
+        <v>2661.78</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>2000</v>
@@ -3756,7 +3756,7 @@
         <v>31011.48</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>0</v>
+        <v>2661.78</v>
       </c>
       <c r="G37" s="6" t="n">
         <v>35500</v>
@@ -3781,7 +3781,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4071,13 +4071,13 @@
         <v>1600</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>-253.02</v>
+        <v>127.14</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>1853.02</v>
+        <v>1472.86</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>-0.1581375</v>
+        <v>0.07946250000000001</v>
       </c>
     </row>
     <row r="13">
@@ -4095,13 +4095,13 @@
         <v>29057</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0</v>
+        <v>2281.62</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>29057</v>
+        <v>26775.38</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0</v>
+        <v>0.07852221495680903</v>
       </c>
     </row>
     <row r="14">
@@ -4138,13 +4138,13 @@
         <v>35184.963</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>-253.02</v>
+        <v>2408.76</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>35437.983</v>
+        <v>32776.203</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>-0.007191140146999728</v>
+        <v>0.0684599270432656</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-24 10:30:24
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -3334,7 +3334,7 @@
         <v>27</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0</v>
+        <v>133.81</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>2500</v>
@@ -3756,7 +3756,7 @@
         <v>31011.48</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>2643.95</v>
+        <v>2777.76</v>
       </c>
       <c r="G37" s="6" t="n">
         <v>35500</v>
@@ -4047,13 +4047,13 @@
         <v>350</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0</v>
+        <v>133.81</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>350</v>
+        <v>216.19</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0</v>
+        <v>0.3823142857142857</v>
       </c>
     </row>
     <row r="12">
@@ -4138,13 +4138,13 @@
         <v>35184.963</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>2390.93</v>
+        <v>2524.74</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>32794.033</v>
+        <v>32660.223</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.06795317647484807</v>
+        <v>0.07175622154270844</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-24 10:30:23
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -1737,10 +1737,10 @@
         <v>0</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>0</v>
+        <v>685.84</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>0</v>
+        <v>5802.81</v>
       </c>
       <c r="N21" s="2" t="n">
         <v>0</v>
@@ -2706,12 +2706,12 @@
       </c>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>0 de 35</t>
+          <t>1 de 35</t>
         </is>
       </c>
       <c r="M37" s="4" t="inlineStr">
         <is>
-          <t>2 de 35</t>
+          <t>3 de 35</t>
         </is>
       </c>
       <c r="N37" s="4" t="inlineStr">
@@ -3334,7 +3334,7 @@
         <v>133.81</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0</v>
+        <v>6488.65</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>0</v>
@@ -3756,7 +3756,7 @@
         <v>14335.17</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>7774.219999999999</v>
+        <v>14262.87</v>
       </c>
       <c r="G37" s="6" t="n">
         <v>2000</v>
@@ -4047,13 +4047,13 @@
         <v>2105</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0</v>
+        <v>685.84</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2105</v>
+        <v>1419.16</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0</v>
+        <v>0.3258147268408551</v>
       </c>
     </row>
     <row r="12">
@@ -4071,13 +4071,13 @@
         <v>25250</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>4105.55</v>
+        <v>9908.360000000001</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>21144.45</v>
+        <v>15341.64</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.1625960396039604</v>
+        <v>0.392410297029703</v>
       </c>
     </row>
     <row r="13">
@@ -4138,13 +4138,13 @@
         <v>30830.233</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>7774.22</v>
+        <v>14262.87</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>23056.013</v>
+        <v>16567.363</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.2521622201168574</v>
+        <v>0.4626260852456094</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-30 10:30:21
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -1740,7 +1740,7 @@
         <v>685.84</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>5735.46</v>
+        <v>9611.620000000001</v>
       </c>
       <c r="N21" s="2" t="n">
         <v>0</v>
@@ -2759,7 +2759,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3334,7 +3334,7 @@
         <v>133.81</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>6421.3</v>
+        <v>10297.46</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>0</v>
@@ -3756,7 +3756,7 @@
         <v>14335.17</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>16016.24</v>
+        <v>19892.4</v>
       </c>
       <c r="G37" s="6" t="n">
         <v>2000</v>
@@ -4071,13 +4071,13 @@
         <v>25250</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>10702.71</v>
+        <v>14578.87</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>14547.29</v>
+        <v>10671.13</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.423869702970297</v>
+        <v>0.5773809900990099</v>
       </c>
     </row>
     <row r="13">
@@ -4138,13 +4138,13 @@
         <v>30830.233</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>16016.24</v>
+        <v>19892.4</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>14813.993</v>
+        <v>10937.833</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.5194978578332509</v>
+        <v>0.6452237970436357</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-05-04 16:30:21
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -993,7 +993,7 @@
         <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0</v>
+        <v>1306.37</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0</v>
@@ -1020,7 +1020,7 @@
         <v>0</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>0</v>
+        <v>6387.62</v>
       </c>
       <c r="N9" s="2" t="n">
         <v>0</v>
@@ -1260,7 +1260,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>0</v>
+        <v>6259.72</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
@@ -2666,52 +2666,52 @@
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
+          <t>1 de 35</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
           <t>0 de 35</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="F37" s="4" t="inlineStr">
         <is>
           <t>0 de 35</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr">
+      <c r="G37" s="4" t="inlineStr">
         <is>
           <t>0 de 35</t>
         </is>
       </c>
-      <c r="G37" s="4" t="inlineStr">
+      <c r="H37" s="4" t="inlineStr">
         <is>
           <t>0 de 35</t>
         </is>
       </c>
-      <c r="H37" s="4" t="inlineStr">
+      <c r="I37" s="4" t="inlineStr">
         <is>
           <t>0 de 35</t>
         </is>
       </c>
-      <c r="I37" s="4" t="inlineStr">
+      <c r="J37" s="4" t="inlineStr">
         <is>
           <t>0 de 35</t>
         </is>
       </c>
-      <c r="J37" s="4" t="inlineStr">
+      <c r="K37" s="4" t="inlineStr">
         <is>
           <t>0 de 35</t>
         </is>
       </c>
-      <c r="K37" s="4" t="inlineStr">
+      <c r="L37" s="4" t="inlineStr">
         <is>
           <t>0 de 35</t>
         </is>
       </c>
-      <c r="L37" s="4" t="inlineStr">
-        <is>
-          <t>0 de 35</t>
-        </is>
-      </c>
       <c r="M37" s="4" t="inlineStr">
         <is>
-          <t>0 de 35</t>
+          <t>2 de 35</t>
         </is>
       </c>
       <c r="N37" s="4" t="inlineStr">
@@ -2759,7 +2759,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3010,7 +3010,7 @@
         <v>7743.69</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0</v>
+        <v>7693.99</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>0</v>
@@ -3118,7 +3118,7 @@
         <v>0</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0</v>
+        <v>6259.72</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>0</v>
@@ -3756,7 +3756,7 @@
         <v>19892.4</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>0</v>
+        <v>13953.71</v>
       </c>
       <c r="G37" s="6" t="n">
         <v>2000</v>

</xml_diff>

<commit_message>
Actualización automática 2026-05-20 12:30:20
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -900,7 +900,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>0</v>
+        <v>13558.54</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -2891,7 +2891,7 @@
       </c>
       <c r="M40" s="4" t="inlineStr">
         <is>
-          <t>4 de 38</t>
+          <t>5 de 38</t>
         </is>
       </c>
       <c r="N40" s="4" t="inlineStr">
@@ -2939,7 +2939,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3190,7 +3190,7 @@
         <v>874.77</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0</v>
+        <v>13558.54</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>0</v>
@@ -4287,7 +4287,7 @@
         <v>19892.4</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>24351.51</v>
+        <v>37910.05</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>2000</v>
@@ -4311,7 +4311,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -4602,13 +4602,13 @@
         <v>44099</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>22597.04</v>
+        <v>36155.58</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>21501.96</v>
+        <v>7943.419999999998</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.5124161545613279</v>
+        <v>0.8198730129934919</v>
       </c>
     </row>
     <row r="13">
@@ -4645,13 +4645,13 @@
         <v>48986.5</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>24351.51</v>
+        <v>37910.05</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>24634.99</v>
+        <v>11076.45</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.4971065497637104</v>
+        <v>0.7738877037551163</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-01 09:30:16
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -455,7 +455,7 @@
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
     <col width="25" customWidth="1" min="11" max="11"/>
     <col width="24" customWidth="1" min="12" max="12"/>
     <col width="17" customWidth="1" min="13" max="13"/>
@@ -891,7 +891,7 @@
         <v>0</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>0</v>
+        <v>104.56</v>
       </c>
       <c r="K7" s="2" t="n">
         <v>0</v>
@@ -2936,7 +2936,7 @@
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>0 de 39</t>
+          <t>1 de 39</t>
         </is>
       </c>
       <c r="K41" s="4" t="inlineStr">
@@ -2999,7 +2999,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3223,7 +3223,7 @@
         <v>1654.08</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0</v>
+        <v>104.56</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>1654</v>
@@ -4050,7 +4050,7 @@
         <v>37855.35</v>
       </c>
       <c r="F39" s="6" t="n">
-        <v>0</v>
+        <v>104.56</v>
       </c>
       <c r="G39" s="6" t="n">
         <v>13854</v>

</xml_diff>

<commit_message>
Actualización automática 2026-07-07 15:30:15
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -1020,7 +1020,7 @@
         <v>0</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>0</v>
+        <v>-15.61</v>
       </c>
       <c r="N9" s="2" t="n">
         <v>0</v>
@@ -3277,7 +3277,7 @@
         <v>7410.07</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0</v>
+        <v>-15.61</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>5390</v>
@@ -4050,7 +4050,7 @@
         <v>37855.35</v>
       </c>
       <c r="F39" s="6" t="n">
-        <v>104.56</v>
+        <v>88.95</v>
       </c>
       <c r="G39" s="6" t="n">
         <v>13854</v>

</xml_diff>

<commit_message>
Actualización automática 2026-07-13 09:30:17
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -900,7 +900,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>0</v>
+        <v>1674.18</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -2951,7 +2951,7 @@
       </c>
       <c r="M41" s="4" t="inlineStr">
         <is>
-          <t>0 de 39</t>
+          <t>1 de 39</t>
         </is>
       </c>
       <c r="N41" s="4" t="inlineStr">
@@ -2999,7 +2999,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3223,7 +3223,7 @@
         <v>1654.08</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>104.56</v>
+        <v>1778.74</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>1654</v>
@@ -4050,7 +4050,7 @@
         <v>37855.35</v>
       </c>
       <c r="F39" s="6" t="n">
-        <v>88.95</v>
+        <v>1763.13</v>
       </c>
       <c r="G39" s="6" t="n">
         <v>13854</v>

</xml_diff>

<commit_message>
Actualización automática 2026-07-13 12:30:16
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -876,7 +876,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0</v>
+        <v>832.61</v>
       </c>
       <c r="F7" s="2" t="n">
         <v>0</v>
@@ -900,7 +900,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>1674.18</v>
+        <v>5783.14</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -2514,7 +2514,7 @@
         <v>0</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>0</v>
+        <v>243.65</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>0</v>
@@ -2911,29 +2911,29 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
+          <t>1 de 39</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
           <t>0 de 39</t>
         </is>
       </c>
-      <c r="F41" s="4" t="inlineStr">
+      <c r="G41" s="4" t="inlineStr">
         <is>
           <t>0 de 39</t>
         </is>
       </c>
-      <c r="G41" s="4" t="inlineStr">
+      <c r="H41" s="4" t="inlineStr">
         <is>
           <t>0 de 39</t>
         </is>
       </c>
-      <c r="H41" s="4" t="inlineStr">
+      <c r="I41" s="4" t="inlineStr">
         <is>
           <t>0 de 39</t>
         </is>
       </c>
-      <c r="I41" s="4" t="inlineStr">
-        <is>
-          <t>0 de 39</t>
-        </is>
-      </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
           <t>1 de 39</t>
@@ -2941,7 +2941,7 @@
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t>0 de 39</t>
+          <t>1 de 39</t>
         </is>
       </c>
       <c r="L41" s="4" t="inlineStr">
@@ -3223,7 +3223,7 @@
         <v>1654.08</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>1778.74</v>
+        <v>6720.31</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>1654</v>
@@ -3844,7 +3844,7 @@
         <v>0</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0</v>
+        <v>243.65</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>0</v>
@@ -4050,7 +4050,7 @@
         <v>37855.35</v>
       </c>
       <c r="F39" s="6" t="n">
-        <v>1763.13</v>
+        <v>6948.35</v>
       </c>
       <c r="G39" s="6" t="n">
         <v>13854</v>

</xml_diff>

<commit_message>
Actualización automática 2026-07-21 15:30:20
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -1920,7 +1920,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>0</v>
+        <v>15.24</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -2951,7 +2951,7 @@
       </c>
       <c r="M41" s="4" t="inlineStr">
         <is>
-          <t>1 de 39</t>
+          <t>2 de 39</t>
         </is>
       </c>
       <c r="N41" s="4" t="inlineStr">
@@ -3628,7 +3628,7 @@
         <v>204.88</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0</v>
+        <v>15.24</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>131</v>
@@ -4050,7 +4050,7 @@
         <v>37855.35</v>
       </c>
       <c r="F39" s="6" t="n">
-        <v>6948.35</v>
+        <v>6963.59</v>
       </c>
       <c r="G39" s="6" t="n">
         <v>13854</v>
@@ -4365,13 +4365,13 @@
         <v>29057</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>5767.53</v>
+        <v>5782.77</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>23289.47</v>
+        <v>23274.23</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.1984902088997487</v>
+        <v>0.1990146952541556</v>
       </c>
     </row>
     <row r="13">
@@ -4408,13 +4408,13 @@
         <v>34944.963</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>6948.35</v>
+        <v>6963.59</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>27996.613</v>
+        <v>27981.373</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.1988369539838975</v>
+        <v>0.1992730683389191</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-03 17:30:16
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -1020,7 +1020,7 @@
         <v>0</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>0</v>
+        <v>8313.379999999999</v>
       </c>
       <c r="N9" s="2" t="n">
         <v>0</v>
@@ -2951,7 +2951,7 @@
       </c>
       <c r="M41" s="4" t="inlineStr">
         <is>
-          <t>0 de 39</t>
+          <t>1 de 39</t>
         </is>
       </c>
       <c r="N41" s="4" t="inlineStr">
@@ -2999,7 +2999,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3277,7 +3277,7 @@
         <v>8184.38</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0</v>
+        <v>8313.379999999999</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>5390</v>
@@ -4050,7 +4050,7 @@
         <v>40935.59</v>
       </c>
       <c r="F39" s="6" t="n">
-        <v>0</v>
+        <v>8313.379999999999</v>
       </c>
       <c r="G39" s="6" t="n">
         <v>13854</v>

</xml_diff>

<commit_message>
Actualización automática 2026-08-05 08:30:16
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R41"/>
+  <dimension ref="A1:R40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>INTROMEX S.A.</t>
+          <t>ITURRALDE ROSALES FRANKLIN DAVID</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ITURRALDE ROSALES FRANKLIN DAVID</t>
+          <t>LINDAO MEJIA FERNANDO AGUILUCHO</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>LINDAO MEJIA FERNANDO AGUILUCHO</t>
+          <t>LINDAO ZUÑIGA BRYAN JOSE</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2306,7 +2306,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>LINDAO ZUÑIGA BRYAN JOSE</t>
+          <t>LUI WONG ANGEL BOLIVAR</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2366,7 +2366,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>LUI WONG ANGEL BOLIVAR</t>
+          <t>MINUTOCORP S.A.</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MINUTOCORP S.A.</t>
+          <t>MUÑOZ FALCONES SERGIO BACILIO</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MUÑOZ FALCONES SERGIO BACILIO</t>
+          <t>PUCO TOAPANTA MARCO ANTONIO</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PUCO TOAPANTA MARCO ANTONIO</t>
+          <t>SANCHEZ BAJANA FRAK XAVIER</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2606,7 +2606,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>SANCHEZ BAJANA FRAK XAVIER</t>
+          <t>SANCHEZ CORREA WILSON SERGIO</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2666,7 +2666,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>SANCHEZ CORREA WILSON SERGIO</t>
+          <t>SOCIEDAD CIVIL Y COMERCIAL GRUPO MOLINA PROAÑO</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2726,7 +2726,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>SOCIEDAD CIVIL Y COMERCIAL GRUPO MOLINA PROAÑO</t>
+          <t>SORIA AVELLAN RAFAEL HUMBERTO</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2786,7 +2786,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SORIA AVELLAN RAFAEL HUMBERTO</t>
+          <t>SOTOMAYOR ORTIZ LUIS JAVIER</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2839,144 +2839,84 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>LINDAO ZUÑIGA BRYAN JOSE</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>SOTOMAYOR ORTIZ LUIS JAVIER</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R40" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>0 de 39</t>
-        </is>
-      </c>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>0 de 39</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="inlineStr">
-        <is>
-          <t>0 de 39</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>0 de 39</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="inlineStr">
-        <is>
-          <t>0 de 39</t>
-        </is>
-      </c>
-      <c r="H41" s="4" t="inlineStr">
-        <is>
-          <t>0 de 39</t>
-        </is>
-      </c>
-      <c r="I41" s="4" t="inlineStr">
-        <is>
-          <t>0 de 39</t>
-        </is>
-      </c>
-      <c r="J41" s="4" t="inlineStr">
-        <is>
-          <t>0 de 39</t>
-        </is>
-      </c>
-      <c r="K41" s="4" t="inlineStr">
-        <is>
-          <t>0 de 39</t>
-        </is>
-      </c>
-      <c r="L41" s="4" t="inlineStr">
-        <is>
-          <t>0 de 39</t>
-        </is>
-      </c>
-      <c r="M41" s="4" t="inlineStr">
-        <is>
-          <t>1 de 39</t>
-        </is>
-      </c>
-      <c r="N41" s="4" t="inlineStr">
-        <is>
-          <t>0 de 39</t>
-        </is>
-      </c>
-      <c r="O41" s="4" t="inlineStr">
-        <is>
-          <t>0 de 39</t>
-        </is>
-      </c>
-      <c r="P41" s="4" t="inlineStr">
-        <is>
-          <t>0 de 39</t>
-        </is>
-      </c>
-      <c r="Q41" s="4" t="inlineStr">
-        <is>
-          <t>0 de 39</t>
-        </is>
-      </c>
-      <c r="R41" s="4" t="inlineStr">
-        <is>
-          <t>0 de 39</t>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>0 de 38</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>0 de 38</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>0 de 38</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>0 de 38</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>0 de 38</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>0 de 38</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>0 de 38</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>0 de 38</t>
+        </is>
+      </c>
+      <c r="K40" s="4" t="inlineStr">
+        <is>
+          <t>0 de 38</t>
+        </is>
+      </c>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>0 de 38</t>
+        </is>
+      </c>
+      <c r="M40" s="4" t="inlineStr">
+        <is>
+          <t>1 de 38</t>
+        </is>
+      </c>
+      <c r="N40" s="4" t="inlineStr">
+        <is>
+          <t>0 de 38</t>
+        </is>
+      </c>
+      <c r="O40" s="4" t="inlineStr">
+        <is>
+          <t>0 de 38</t>
+        </is>
+      </c>
+      <c r="P40" s="4" t="inlineStr">
+        <is>
+          <t>0 de 38</t>
+        </is>
+      </c>
+      <c r="Q40" s="4" t="inlineStr">
+        <is>
+          <t>0 de 38</t>
+        </is>
+      </c>
+      <c r="R40" s="4" t="inlineStr">
+        <is>
+          <t>0 de 38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-08-07 12:30:15
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -597,7 +597,7 @@
         <v>0</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>0</v>
+        <v>457.23</v>
       </c>
       <c r="M2" s="2" t="n">
         <v>0</v>
@@ -2886,7 +2886,7 @@
       </c>
       <c r="L40" s="4" t="inlineStr">
         <is>
-          <t>0 de 38</t>
+          <t>1 de 38</t>
         </is>
       </c>
       <c r="M40" s="4" t="inlineStr">
@@ -3001,7 +3001,7 @@
         <v>0</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0</v>
+        <v>457.23</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>1166</v>
@@ -3990,7 +3990,7 @@
         <v>40935.59</v>
       </c>
       <c r="F39" s="6" t="n">
-        <v>8158.419999999999</v>
+        <v>8615.65</v>
       </c>
       <c r="G39" s="6" t="n">
         <v>13854</v>

</xml_diff>

<commit_message>
Actualización automática 2026-08-31 11:30:22
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -876,7 +876,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0</v>
+        <v>394.76</v>
       </c>
       <c r="F7" s="2" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
         <v>0</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>0</v>
+        <v>108.29</v>
       </c>
       <c r="L7" s="2" t="n">
         <v>0</v>
@@ -2454,7 +2454,7 @@
         <v>0</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>81.22</v>
+        <v>270.66</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>0</v>
@@ -2851,37 +2851,37 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
+          <t>1 de 38</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
           <t>0 de 38</t>
         </is>
       </c>
-      <c r="F40" s="4" t="inlineStr">
+      <c r="G40" s="4" t="inlineStr">
         <is>
           <t>0 de 38</t>
         </is>
       </c>
-      <c r="G40" s="4" t="inlineStr">
+      <c r="H40" s="4" t="inlineStr">
         <is>
           <t>0 de 38</t>
         </is>
       </c>
-      <c r="H40" s="4" t="inlineStr">
+      <c r="I40" s="4" t="inlineStr">
         <is>
           <t>0 de 38</t>
         </is>
       </c>
-      <c r="I40" s="4" t="inlineStr">
+      <c r="J40" s="4" t="inlineStr">
         <is>
           <t>0 de 38</t>
         </is>
       </c>
-      <c r="J40" s="4" t="inlineStr">
-        <is>
-          <t>0 de 38</t>
-        </is>
-      </c>
       <c r="K40" s="4" t="inlineStr">
         <is>
-          <t>2 de 38</t>
+          <t>3 de 38</t>
         </is>
       </c>
       <c r="L40" s="4" t="inlineStr">
@@ -3163,7 +3163,7 @@
         <v>13787.67</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>-141.44</v>
+        <v>361.61</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>1654</v>
@@ -3784,7 +3784,7 @@
         <v>1327.27</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>81.22</v>
+        <v>270.66</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>0</v>
@@ -3990,7 +3990,7 @@
         <v>40935.59</v>
       </c>
       <c r="F39" s="6" t="n">
-        <v>12178.56</v>
+        <v>12871.05</v>
       </c>
       <c r="G39" s="6" t="n">
         <v>13854</v>
@@ -4113,13 +4113,13 @@
         <v>199.5</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0</v>
+        <v>394.76</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>199.5</v>
+        <v>-195.26</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0</v>
+        <v>1.97874686716792</v>
       </c>
     </row>
     <row r="5">
@@ -4233,13 +4233,13 @@
         <v>203.763</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>3118.38</v>
+        <v>3416.11</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-2914.617</v>
+        <v>-3212.347</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>15.30395606660679</v>
+        <v>16.76511437307068</v>
       </c>
     </row>
     <row r="10">
@@ -4348,13 +4348,13 @@
         <v>40761.643</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>12178.56</v>
+        <v>12871.05</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>28583.083</v>
+        <v>27890.593</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.2987750027642408</v>
+        <v>0.3157637684035454</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-08 17:30:17
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -840,7 +840,7 @@
         <v>0</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>0</v>
+        <v>1338.48</v>
       </c>
       <c r="N6" s="2" t="n">
         <v>0</v>
@@ -2625,7 +2625,7 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>0</v>
+        <v>782.1</v>
       </c>
       <c r="I36" s="2" t="n">
         <v>0</v>
@@ -2637,10 +2637,10 @@
         <v>0</v>
       </c>
       <c r="L36" s="2" t="n">
-        <v>0</v>
+        <v>479.69</v>
       </c>
       <c r="M36" s="2" t="n">
-        <v>0</v>
+        <v>1344.33</v>
       </c>
       <c r="N36" s="2" t="n">
         <v>0</v>
@@ -2806,32 +2806,32 @@
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
+          <t>1 de 37</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
           <t>0 de 37</t>
         </is>
       </c>
-      <c r="I39" s="4" t="inlineStr">
+      <c r="J39" s="4" t="inlineStr">
         <is>
           <t>0 de 37</t>
         </is>
       </c>
-      <c r="J39" s="4" t="inlineStr">
+      <c r="K39" s="4" t="inlineStr">
         <is>
           <t>0 de 37</t>
         </is>
       </c>
-      <c r="K39" s="4" t="inlineStr">
-        <is>
-          <t>0 de 37</t>
-        </is>
-      </c>
       <c r="L39" s="4" t="inlineStr">
         <is>
-          <t>0 de 37</t>
+          <t>1 de 37</t>
         </is>
       </c>
       <c r="M39" s="4" t="inlineStr">
         <is>
-          <t>0 de 37</t>
+          <t>2 de 37</t>
         </is>
       </c>
       <c r="N39" s="4" t="inlineStr">
@@ -3022,7 +3022,7 @@
         <v>0</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0</v>
+        <v>1338.48</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>2500</v>
@@ -3751,7 +3751,7 @@
         <v>2127.79</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0</v>
+        <v>2606.12</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>2000</v>
@@ -3768,7 +3768,7 @@
         <v>39346.94</v>
       </c>
       <c r="F33" s="6" t="n">
-        <v>-54.81</v>
+        <v>3889.79</v>
       </c>
       <c r="G33" s="6" t="n">
         <v>39500</v>
@@ -3793,7 +3793,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3963,13 +3963,13 @@
         <v>615</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0</v>
+        <v>782.1</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>615</v>
+        <v>-167.1</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0</v>
+        <v>1.271707317073171</v>
       </c>
     </row>
     <row r="8">
@@ -4107,13 +4107,13 @@
         <v>970</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0</v>
+        <v>479.69</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>970</v>
+        <v>490.31</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0</v>
+        <v>0.4945257731958763</v>
       </c>
     </row>
     <row r="14">
@@ -4131,13 +4131,13 @@
         <v>35464</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>-54.81</v>
+        <v>2628</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>35518.81</v>
+        <v>32836</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>-0.001545510940672231</v>
+        <v>0.07410331603879991</v>
       </c>
     </row>
     <row r="15">
@@ -4174,13 +4174,13 @@
         <v>45197.643</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>-54.81</v>
+        <v>3889.79</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>45252.453</v>
+        <v>41307.853</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>-0.001212673855581363</v>
+        <v>0.08606178866451066</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-11 09:30:18
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -455,7 +455,7 @@
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
     <col width="25" customWidth="1" min="11" max="11"/>
     <col width="24" customWidth="1" min="12" max="12"/>
     <col width="17" customWidth="1" min="13" max="13"/>
@@ -891,7 +891,7 @@
         <v>0</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>0</v>
+        <v>104.56</v>
       </c>
       <c r="K7" s="2" t="n">
         <v>0</v>
@@ -2280,7 +2280,7 @@
         <v>0</v>
       </c>
       <c r="M30" s="2" t="n">
-        <v>0</v>
+        <v>37.08</v>
       </c>
       <c r="N30" s="2" t="n">
         <v>0</v>
@@ -2816,14 +2816,14 @@
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
+          <t>1 de 37</t>
+        </is>
+      </c>
+      <c r="K39" s="4" t="inlineStr">
+        <is>
           <t>0 de 37</t>
         </is>
       </c>
-      <c r="K39" s="4" t="inlineStr">
-        <is>
-          <t>0 de 37</t>
-        </is>
-      </c>
       <c r="L39" s="4" t="inlineStr">
         <is>
           <t>1 de 37</t>
@@ -2831,7 +2831,7 @@
       </c>
       <c r="M39" s="4" t="inlineStr">
         <is>
-          <t>2 de 37</t>
+          <t>3 de 37</t>
         </is>
       </c>
       <c r="N39" s="4" t="inlineStr">
@@ -3076,7 +3076,7 @@
         <v>22863.45</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>-54.81</v>
+        <v>49.75</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>8000</v>
@@ -3768,7 +3768,7 @@
         <v>39346.94</v>
       </c>
       <c r="F33" s="6" t="n">
-        <v>3889.79</v>
+        <v>3994.35</v>
       </c>
       <c r="G33" s="6" t="n">
         <v>39500</v>
@@ -3791,7 +3791,7 @@
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
@@ -4035,10 +4035,10 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0</v>
+        <v>104.56</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0</v>
+        <v>-104.56</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>0</v>
@@ -4131,13 +4131,13 @@
         <v>35464</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>2628</v>
+        <v>2665.08</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>32836</v>
+        <v>32798.92</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.07410331603879991</v>
+        <v>0.07514888337468982</v>
       </c>
     </row>
     <row r="15">
@@ -4174,13 +4174,13 @@
         <v>45197.643</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>3889.79</v>
+        <v>4031.43</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>41307.853</v>
+        <v>41166.213</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.08606178866451066</v>
+        <v>0.08919558039785393</v>
       </c>
     </row>
   </sheetData>

</xml_diff>